<commit_message>
Actualizar datos.xlsx con datos corregidos YTD Mayo 2026
Total trabajos: 517 → 616 (+99 trabajos, +19%)
Total horas: 3.053h → 3.924h (+871h, +29%)
Retail: nueva categoría con volumen significativo (99 proyectos, 748h)
Entrega: nueva estructura con desglose Bdesign/Retail (media 1.96d vs 2.15d)
RRSS: 94 → 97 publicaciones, 73h → 126h
Actualiza parseExcel para leer hoja Entrega con múltiples categorías

https://claude.ai/code/session_01A4SLDFHLc22bTWoXT2NUrv
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscar.nieto/Desktop/T/BDESIGN/DASHBOARD/__INTERACTIVO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://savillsglobal-my.sharepoint.com/personal/oscar_nieto_savills_es/Documents/Archivos de chat de Microsoft Teams/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A89D243B-7CED-E64E-BDFF-E29013313185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="132" documentId="13_ncr:1_{A89D243B-7CED-E64E-BDFF-E29013313185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94ADA68F-4576-43E6-92A7-705F8C539229}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="3264" yWindow="2664" windowWidth="17436" windowHeight="9756" tabRatio="500" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="111">
   <si>
     <t>PLANTILLA DASHBOARD BDESIGN</t>
   </si>
@@ -252,9 +252,6 @@
     <t>Métrica</t>
   </si>
   <si>
-    <t>Días medios de entrega</t>
-  </si>
-  <si>
     <t>MEDIA YTD</t>
   </si>
   <si>
@@ -376,6 +373,9 @@
   </si>
   <si>
     <t>Sevilla</t>
+  </si>
+  <si>
+    <t>Bdesign</t>
   </si>
 </sst>
 </file>
@@ -524,14 +524,14 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -620,6 +620,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -802,262 +806,277 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D37"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="4" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="23" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:4" ht="22.8" x14ac:dyDescent="0.4">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-    </row>
-    <row r="3" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+    </row>
+    <row r="3" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-    </row>
-    <row r="6" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+    </row>
+    <row r="6" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-    </row>
-    <row r="7" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+    </row>
+    <row r="7" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-    </row>
-    <row r="9" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+    </row>
+    <row r="9" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-    </row>
-    <row r="12" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+    </row>
+    <row r="12" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-    </row>
-    <row r="13" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+    </row>
+    <row r="13" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-    </row>
-    <row r="14" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+    </row>
+    <row r="14" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-    </row>
-    <row r="15" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+    </row>
+    <row r="15" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-    </row>
-    <row r="16" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+    </row>
+    <row r="16" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="15" t="s">
+      <c r="B16" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-    </row>
-    <row r="17" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+    </row>
+    <row r="17" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="15" t="s">
+      <c r="B17" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-    </row>
-    <row r="20" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+    </row>
+    <row r="20" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="15" t="s">
+      <c r="B22" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-    </row>
-    <row r="23" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+    </row>
+    <row r="23" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="B23" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-    </row>
-    <row r="24" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+    </row>
+    <row r="24" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-    </row>
-    <row r="25" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+    </row>
+    <row r="25" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-    </row>
-    <row r="26" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+    </row>
+    <row r="26" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B26" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-    </row>
-    <row r="29" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+    </row>
+    <row r="29" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-    </row>
-    <row r="32" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+    </row>
+    <row r="32" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="15" t="s">
+      <c r="B32" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-    </row>
-    <row r="33" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+    </row>
+    <row r="33" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B33" s="15" t="s">
+      <c r="B33" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C33" s="15"/>
-      <c r="D33" s="15"/>
-    </row>
-    <row r="34" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+    </row>
+    <row r="34" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B34" s="15" t="s">
+      <c r="B34" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-    </row>
-    <row r="35" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+    </row>
+    <row r="35" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B35" s="15" t="s">
+      <c r="B35" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-    </row>
-    <row r="36" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+    </row>
+    <row r="36" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B36" s="15" t="s">
+      <c r="B36" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
-    </row>
-    <row r="37" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+    </row>
+    <row r="37" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B37" s="15" t="s">
+      <c r="B37" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C37" s="15"/>
-      <c r="D37" s="15"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B25:D25"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="B37:D37"/>
@@ -1066,21 +1085,6 @@
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1090,13 +1094,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>47</v>
       </c>
@@ -1107,78 +1111,86 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>48</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>50</v>
       </c>
       <c r="B4" s="8">
-        <v>23</v>
+        <f>23+7</f>
+        <v>30</v>
       </c>
       <c r="C4" s="8">
-        <v>28</v>
+        <f>28+10</f>
+        <v>38</v>
       </c>
       <c r="D4" s="8">
-        <v>23</v>
+        <f>23+8</f>
+        <v>31</v>
       </c>
       <c r="E4" s="8">
-        <v>25</v>
+        <f>25+9</f>
+        <v>34</v>
       </c>
       <c r="F4" s="8">
-        <v>38</v>
+        <f>38+8</f>
+        <v>46</v>
       </c>
       <c r="G4" s="9">
-        <f>SUM(B4:F4)</f>
-        <v>137</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" ref="G4:G18" si="0">SUM(B4:F4)</f>
+        <v>179</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>45</v>
       </c>
       <c r="B5" s="8">
-        <v>25</v>
+        <f>25+1</f>
+        <v>26</v>
       </c>
       <c r="C5" s="8">
         <v>21</v>
       </c>
       <c r="D5" s="8">
-        <v>22</v>
+        <f>22+1</f>
+        <v>23</v>
       </c>
       <c r="E5" s="8">
-        <v>7</v>
+        <f>7+1</f>
+        <v>8</v>
       </c>
       <c r="F5" s="8">
         <v>20</v>
       </c>
       <c r="G5" s="9">
-        <f>SUM(B5:F5)</f>
-        <v>95</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>51</v>
       </c>
@@ -1192,52 +1204,62 @@
         <v>12</v>
       </c>
       <c r="E6" s="8">
-        <v>13</v>
+        <f>13+2</f>
+        <v>15</v>
       </c>
       <c r="F6" s="8">
-        <v>18</v>
+        <f>18+1</f>
+        <v>19</v>
       </c>
       <c r="G6" s="9">
-        <f>SUM(B6:F6)</f>
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B7" s="8">
+        <f>14+2</f>
+        <v>16</v>
+      </c>
+      <c r="C7" s="8">
+        <f>8+6</f>
         <v>14</v>
       </c>
-      <c r="C7" s="8">
-        <v>8</v>
-      </c>
       <c r="D7" s="8">
-        <v>11</v>
+        <f>11+3</f>
+        <v>14</v>
       </c>
       <c r="E7" s="8">
-        <v>11</v>
+        <f>11+10</f>
+        <v>21</v>
       </c>
       <c r="F7" s="8">
-        <v>12</v>
+        <f>12+4</f>
+        <v>16</v>
       </c>
       <c r="G7" s="9">
-        <f>SUM(B7:F7)</f>
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>52</v>
       </c>
       <c r="B8" s="8">
+        <f>9+1</f>
+        <v>10</v>
+      </c>
+      <c r="C8" s="8">
+        <f>6+1</f>
+        <v>7</v>
+      </c>
+      <c r="D8" s="8">
+        <f>7+2</f>
         <v>9</v>
-      </c>
-      <c r="C8" s="8">
-        <v>6</v>
-      </c>
-      <c r="D8" s="8">
-        <v>7</v>
       </c>
       <c r="E8" s="8">
         <v>11</v>
@@ -1246,13 +1268,13 @@
         <v>3</v>
       </c>
       <c r="G8" s="9">
-        <f>SUM(B8:F8)</f>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B9" s="8">
         <v>5</v>
@@ -1270,13 +1292,13 @@
         <v>3</v>
       </c>
       <c r="G9" s="9">
-        <f>SUM(B9:F9)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B10" s="8">
         <v>3</v>
@@ -1294,37 +1316,42 @@
         <v>8</v>
       </c>
       <c r="G10" s="9">
-        <f>SUM(B10:F10)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B11" s="8">
-        <v>9</v>
+        <f>9+1</f>
+        <v>10</v>
       </c>
       <c r="C11" s="8">
+        <f>4+6</f>
+        <v>10</v>
+      </c>
+      <c r="D11" s="8">
+        <f>4+3</f>
+        <v>7</v>
+      </c>
+      <c r="E11" s="8">
+        <f>3+2</f>
+        <v>5</v>
+      </c>
+      <c r="F11" s="8">
+        <f>3+1</f>
         <v>4</v>
       </c>
-      <c r="D11" s="8">
-        <v>4</v>
-      </c>
-      <c r="E11" s="8">
-        <v>3</v>
-      </c>
-      <c r="F11" s="8">
-        <v>3</v>
-      </c>
       <c r="G11" s="9">
-        <f>SUM(B11:F11)</f>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B12" s="8">
         <v>3</v>
@@ -1332,24 +1359,30 @@
       <c r="C12" s="8">
         <v>1</v>
       </c>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
+      <c r="D12" s="8">
+        <v>0</v>
+      </c>
+      <c r="E12" s="8">
+        <v>0</v>
+      </c>
       <c r="F12" s="8">
         <v>7</v>
       </c>
       <c r="G12" s="9">
-        <f>SUM(B12:F12)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>53</v>
       </c>
       <c r="B13" s="8">
         <v>4</v>
       </c>
-      <c r="C13" s="8"/>
+      <c r="C13" s="8">
+        <v>0</v>
+      </c>
       <c r="D13" s="8">
         <v>1</v>
       </c>
@@ -1360,16 +1393,17 @@
         <v>2</v>
       </c>
       <c r="G13" s="9">
-        <f>SUM(B13:F13)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B14" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="C14" s="8">
         <v>2</v>
@@ -1382,93 +1416,113 @@
         <v>2</v>
       </c>
       <c r="G14" s="9">
-        <f>SUM(B14:F14)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B15" s="8">
+        <f>2+1</f>
+        <v>3</v>
+      </c>
+      <c r="C15" s="8">
+        <f>2+1</f>
+        <v>3</v>
+      </c>
+      <c r="D15" s="8">
+        <f>2+1</f>
+        <v>3</v>
+      </c>
+      <c r="E15" s="8">
+        <v>1</v>
+      </c>
+      <c r="F15" s="8">
+        <v>0</v>
+      </c>
+      <c r="G15" s="9">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="8" t="s">
         <v>78</v>
-      </c>
-      <c r="B15" s="8">
-        <v>2</v>
-      </c>
-      <c r="C15" s="8">
-        <v>2</v>
-      </c>
-      <c r="D15" s="8">
-        <v>2</v>
-      </c>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="9">
-        <f>SUM(B15:F15)</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="8" t="s">
-        <v>79</v>
       </c>
       <c r="B16" s="8">
         <v>3</v>
       </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
+      <c r="C16" s="8">
+        <v>0</v>
+      </c>
+      <c r="D16" s="8">
+        <v>2</v>
+      </c>
       <c r="E16" s="8">
         <v>1</v>
       </c>
       <c r="F16" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="G16" s="9">
-        <f>SUM(B16:F16)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
+        <v>81</v>
+      </c>
+      <c r="B17" s="8">
+        <v>0</v>
+      </c>
+      <c r="C17" s="8">
+        <v>0</v>
+      </c>
+      <c r="D17" s="8">
+        <v>1</v>
+      </c>
       <c r="E17" s="8">
         <v>1</v>
       </c>
-      <c r="F17" s="8"/>
+      <c r="F17" s="8">
+        <v>0</v>
+      </c>
       <c r="G17" s="10">
-        <f>SUM(B17:F17)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>54</v>
       </c>
       <c r="B18" s="11">
         <f>SUM(B4:B17)</f>
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C18" s="11">
         <f>SUM(C4:C17)</f>
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="D18" s="11">
         <f>SUM(D4:D17)</f>
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="E18" s="11">
         <f>SUM(E4:E17)</f>
-        <v>89</v>
+        <v>114</v>
       </c>
       <c r="F18" s="11">
         <f>SUM(F4:F17)</f>
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="G18" s="11">
-        <f>SUM(B18:F18)</f>
-        <v>517</v>
+        <f t="shared" si="0"/>
+        <v>616</v>
       </c>
     </row>
   </sheetData>
@@ -1483,13 +1537,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>55</v>
       </c>
@@ -1500,35 +1554,36 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>56</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B4" s="8">
-        <v>26</v>
+        <f>26+1</f>
+        <v>27</v>
       </c>
       <c r="C4" s="8">
         <v>24</v>
@@ -1537,17 +1592,19 @@
         <v>20</v>
       </c>
       <c r="E4" s="8">
+        <f>18+2</f>
+        <v>20</v>
+      </c>
+      <c r="F4" s="8">
+        <f>15+3</f>
         <v>18</v>
       </c>
-      <c r="F4" s="8">
-        <v>15</v>
-      </c>
       <c r="G4" s="8">
-        <f>SUM(B4:F4)</f>
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" ref="G4:G25" si="0">SUM(B4:F4)</f>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>57</v>
       </c>
@@ -1567,13 +1624,13 @@
         <v>36</v>
       </c>
       <c r="G5" s="8">
-        <f>SUM(B5:F5)</f>
+        <f t="shared" si="0"/>
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B6" s="8">
         <v>14</v>
@@ -1591,13 +1648,13 @@
         <v>9</v>
       </c>
       <c r="G6" s="8">
-        <f>SUM(B6:F6)</f>
+        <f t="shared" si="0"/>
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B7" s="8">
         <v>7</v>
@@ -1609,17 +1666,18 @@
         <v>16</v>
       </c>
       <c r="E7" s="8">
-        <v>13</v>
+        <f>13+1</f>
+        <v>14</v>
       </c>
       <c r="F7" s="8">
         <v>1</v>
       </c>
       <c r="G7" s="8">
-        <f>SUM(B7:F7)</f>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>58</v>
       </c>
@@ -1627,7 +1685,8 @@
         <v>10</v>
       </c>
       <c r="C8" s="8">
-        <v>10</v>
+        <f>10+1</f>
+        <v>11</v>
       </c>
       <c r="D8" s="8">
         <v>5</v>
@@ -1639,13 +1698,13 @@
         <v>6</v>
       </c>
       <c r="G8" s="8">
-        <f>SUM(B8:F8)</f>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B9" s="8">
         <v>5</v>
@@ -1663,13 +1722,13 @@
         <v>17</v>
       </c>
       <c r="G9" s="8">
-        <f>SUM(B9:F9)</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B10" s="8">
         <v>12</v>
@@ -1687,22 +1746,24 @@
         <v>3</v>
       </c>
       <c r="G10" s="8">
-        <f>SUM(B10:F10)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B11" s="8">
-        <v>5</v>
+        <f>5+1</f>
+        <v>6</v>
       </c>
       <c r="C11" s="8">
         <v>4</v>
       </c>
       <c r="D11" s="8">
-        <v>5</v>
+        <f>5+2</f>
+        <v>7</v>
       </c>
       <c r="E11" s="8">
         <v>3</v>
@@ -1711,11 +1772,11 @@
         <v>7</v>
       </c>
       <c r="G11" s="8">
-        <f>SUM(B11:F11)</f>
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>60</v>
       </c>
@@ -1735,57 +1796,65 @@
         <v>7</v>
       </c>
       <c r="G12" s="8">
-        <f>SUM(B12:F12)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>59</v>
       </c>
       <c r="B13" s="8">
-        <v>3</v>
+        <f>3+12</f>
+        <v>15</v>
       </c>
       <c r="C13" s="8">
-        <v>2</v>
+        <f>2+23</f>
+        <v>25</v>
       </c>
       <c r="D13" s="8">
-        <v>3</v>
-      </c>
-      <c r="E13" s="8"/>
+        <f>3+18</f>
+        <v>21</v>
+      </c>
+      <c r="E13" s="8">
+        <v>23</v>
+      </c>
       <c r="F13" s="8">
-        <v>2</v>
+        <f>2+13</f>
+        <v>15</v>
       </c>
       <c r="G13" s="8">
-        <f>SUM(B13:F13)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8">
         <v>3</v>
       </c>
       <c r="D14" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="E14" s="8">
         <v>1</v>
       </c>
       <c r="F14" s="8">
-        <v>3</v>
+        <f>3+1</f>
+        <v>4</v>
       </c>
       <c r="G14" s="8">
-        <f>SUM(B14:F14)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8">
@@ -1799,35 +1868,39 @@
         <v>3</v>
       </c>
       <c r="G15" s="8">
-        <f>SUM(B15:F15)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B16" s="8">
-        <v>1</v>
+        <f>1+2</f>
+        <v>3</v>
       </c>
       <c r="C16" s="8">
         <v>2</v>
       </c>
-      <c r="D16" s="8"/>
+      <c r="D16" s="8">
+        <v>2</v>
+      </c>
       <c r="E16" s="8">
         <v>3</v>
       </c>
       <c r="F16" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="G16" s="8">
-        <f>SUM(B16:F16)</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B17" s="8">
         <v>3</v>
@@ -1841,19 +1914,20 @@
         <v>2</v>
       </c>
       <c r="G17" s="8">
-        <f>SUM(B17:F17)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B18" s="8">
         <v>2</v>
       </c>
       <c r="C18" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="D18" s="8">
         <v>1</v>
@@ -1863,13 +1937,13 @@
       </c>
       <c r="F18" s="8"/>
       <c r="G18" s="8">
-        <f>SUM(B18:F18)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="8">
@@ -1883,13 +1957,13 @@
         <v>2</v>
       </c>
       <c r="G19" s="8">
-        <f>SUM(B19:F19)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B20" s="8">
         <v>1</v>
@@ -1905,13 +1979,13 @@
         <v>1</v>
       </c>
       <c r="G20" s="8">
-        <f>SUM(B20:F20)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8">
@@ -1923,13 +1997,13 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
       <c r="G21" s="8">
-        <f>SUM(B21:F21)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -1939,31 +2013,34 @@
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
       <c r="G22" s="8">
-        <f>SUM(B22:F22)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
       <c r="D23" s="8">
         <v>1</v>
       </c>
-      <c r="E23" s="8"/>
+      <c r="E23" s="8">
+        <v>1</v>
+      </c>
       <c r="F23" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="G23" s="8">
-        <f>SUM(B23:F23)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B24" s="8">
         <v>1</v>
@@ -1973,37 +2050,37 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
       <c r="G24" s="8">
-        <f>SUM(B24:F24)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>54</v>
       </c>
       <c r="B25" s="4">
         <f>SUM(B4:B24)</f>
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="C25" s="4">
         <f>SUM(C4:C24)</f>
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="D25" s="4">
         <f>SUM(D4:D24)</f>
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="E25" s="4">
         <f>SUM(E4:E24)</f>
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="F25" s="4">
         <f>SUM(F4:F24)</f>
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="G25" s="4">
-        <f>SUM(B25:F25)</f>
-        <v>517</v>
+        <f t="shared" si="0"/>
+        <v>627</v>
       </c>
     </row>
   </sheetData>
@@ -2018,13 +2095,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>61</v>
       </c>
@@ -2035,35 +2112,36 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>56</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B4" s="8">
-        <v>165.5</v>
+        <f>165.5+0.5</f>
+        <v>166</v>
       </c>
       <c r="C4" s="8">
         <v>279.75</v>
@@ -2078,11 +2156,11 @@
         <v>191</v>
       </c>
       <c r="G4" s="7">
-        <f>SUM(B4:F4)</f>
-        <v>923.25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" ref="G4:G27" si="0">SUM(B4:F4)</f>
+        <v>923.75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>57</v>
       </c>
@@ -2102,13 +2180,13 @@
         <v>110.25</v>
       </c>
       <c r="G5" s="7">
-        <f>SUM(B5:F5)</f>
+        <f t="shared" si="0"/>
         <v>399.55</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B6" s="8">
         <v>26.5</v>
@@ -2120,17 +2198,19 @@
         <v>102.5</v>
       </c>
       <c r="E6" s="8">
-        <v>58</v>
+        <f>58+9.5</f>
+        <v>67.5</v>
       </c>
       <c r="F6" s="8">
-        <v>25.75</v>
+        <f>25.75+7.5</f>
+        <v>33.25</v>
       </c>
       <c r="G6" s="7">
-        <f>SUM(B6:F6)</f>
-        <v>275</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>292</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>58</v>
       </c>
@@ -2138,7 +2218,8 @@
         <v>89</v>
       </c>
       <c r="C7" s="8">
-        <v>65.5</v>
+        <f>65.5+3</f>
+        <v>68.5</v>
       </c>
       <c r="D7" s="8">
         <v>28</v>
@@ -2150,13 +2231,13 @@
         <v>19.75</v>
       </c>
       <c r="G7" s="7">
-        <f>SUM(B7:F7)</f>
-        <v>268.25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>271.25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B8" s="8">
         <v>29.25</v>
@@ -2168,19 +2249,20 @@
         <v>71.5</v>
       </c>
       <c r="E8" s="8">
-        <v>81</v>
+        <f>81+3</f>
+        <v>84</v>
       </c>
       <c r="F8" s="8">
         <v>1</v>
       </c>
       <c r="G8" s="7">
-        <f>SUM(B8:F8)</f>
-        <v>226.25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>229.25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B9" s="8">
         <v>74</v>
@@ -2198,13 +2280,13 @@
         <v>24.75</v>
       </c>
       <c r="G9" s="7">
-        <f>SUM(B9:F9)</f>
+        <f t="shared" si="0"/>
         <v>182.75</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B10" s="8">
         <v>13</v>
@@ -2222,22 +2304,24 @@
         <v>82</v>
       </c>
       <c r="G10" s="7">
-        <f>SUM(B10:F10)</f>
+        <f t="shared" si="0"/>
         <v>171.5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B11" s="8">
-        <v>16.75</v>
+        <f>16.75+20.5</f>
+        <v>37.25</v>
       </c>
       <c r="C11" s="8">
         <v>8</v>
       </c>
       <c r="D11" s="8">
-        <v>38</v>
+        <f>38+31.5</f>
+        <v>69.5</v>
       </c>
       <c r="E11" s="8">
         <v>40.5</v>
@@ -2246,11 +2330,11 @@
         <v>37.5</v>
       </c>
       <c r="G11" s="7">
-        <f>SUM(B11:F11)</f>
-        <v>140.75</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>192.75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>60</v>
       </c>
@@ -2270,13 +2354,13 @@
         <v>32.5</v>
       </c>
       <c r="G12" s="7">
-        <f>SUM(B12:F12)</f>
+        <f t="shared" si="0"/>
         <v>106.75</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B13" s="8">
         <v>9</v>
@@ -2294,13 +2378,13 @@
         <v>5</v>
       </c>
       <c r="G13" s="7">
-        <f>SUM(B13:F13)</f>
+        <f t="shared" si="0"/>
         <v>62.75</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8">
@@ -2314,13 +2398,13 @@
         <v>48</v>
       </c>
       <c r="G14" s="7">
-        <f>SUM(B14:F14)</f>
+        <f t="shared" si="0"/>
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B15" s="8">
         <v>39.5</v>
@@ -2334,13 +2418,13 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="7">
-        <f>SUM(B15:F15)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B16" s="8">
         <v>4.5</v>
@@ -2356,79 +2440,91 @@
         <v>4</v>
       </c>
       <c r="G16" s="7">
-        <f>SUM(B16:F16)</f>
+        <f t="shared" si="0"/>
         <v>27.75</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>59</v>
       </c>
       <c r="B17" s="8">
-        <v>13.5</v>
+        <f>13.5+72.55</f>
+        <v>86.05</v>
       </c>
       <c r="C17" s="8">
-        <v>3.75</v>
+        <f>3.75+240.5</f>
+        <v>244.25</v>
       </c>
       <c r="D17" s="8">
-        <v>5.75</v>
-      </c>
-      <c r="E17" s="8"/>
+        <f>5.75+207.5</f>
+        <v>213.25</v>
+      </c>
+      <c r="E17" s="8">
+        <v>125.25</v>
+      </c>
       <c r="F17" s="8">
-        <v>4</v>
+        <f>4+75</f>
+        <v>79</v>
       </c>
       <c r="G17" s="7">
-        <f>SUM(B17:F17)</f>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>747.8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="8">
         <v>14.5</v>
       </c>
       <c r="D18" s="8">
-        <v>5</v>
+        <f>5+1</f>
+        <v>6</v>
       </c>
       <c r="E18" s="8">
         <v>4</v>
       </c>
       <c r="F18" s="8">
-        <v>3.25</v>
+        <f>3.25+27.5</f>
+        <v>30.75</v>
       </c>
       <c r="G18" s="7">
-        <f>SUM(B18:F18)</f>
-        <v>26.75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>55.25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B19" s="8">
-        <v>3</v>
+        <f>3+22</f>
+        <v>25</v>
       </c>
       <c r="C19" s="8">
         <v>4</v>
       </c>
-      <c r="D19" s="8"/>
+      <c r="D19" s="8">
+        <v>4.25</v>
+      </c>
       <c r="E19" s="8">
         <v>16.75</v>
       </c>
       <c r="F19" s="8">
-        <v>1</v>
+        <f>1+1.25</f>
+        <v>2.25</v>
       </c>
       <c r="G19" s="7">
-        <f>SUM(B19:F19)</f>
-        <v>24.75</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>52.25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -2438,31 +2534,34 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
       <c r="G20" s="7">
-        <f>SUM(B20:F20)</f>
+        <f t="shared" si="0"/>
         <v>24.25</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
       <c r="D21" s="8">
         <v>13</v>
       </c>
-      <c r="E21" s="8"/>
+      <c r="E21" s="8">
+        <v>6</v>
+      </c>
       <c r="F21" s="8">
-        <v>3</v>
+        <f>3+11.5</f>
+        <v>14.5</v>
       </c>
       <c r="G21" s="7">
-        <f>SUM(B21:F21)</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B22" s="8">
         <v>12</v>
@@ -2472,13 +2571,13 @@
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
       <c r="G22" s="7">
-        <f>SUM(B22:F22)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8">
@@ -2490,13 +2589,13 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
       <c r="G23" s="7">
-        <f>SUM(B23:F23)</f>
+        <f t="shared" si="0"/>
         <v>11.5</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8">
@@ -2510,19 +2609,20 @@
         <v>5</v>
       </c>
       <c r="G24" s="7">
-        <f>SUM(B24:F24)</f>
+        <f t="shared" si="0"/>
         <v>9.5</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B25" s="8">
         <v>5</v>
       </c>
       <c r="C25" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="D25" s="8">
         <v>1</v>
@@ -2532,13 +2632,13 @@
       </c>
       <c r="F25" s="8"/>
       <c r="G25" s="7">
-        <f>SUM(B25:F25)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -2548,37 +2648,37 @@
         <v>1</v>
       </c>
       <c r="G26" s="7">
-        <f>SUM(B26:F26)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>54</v>
       </c>
       <c r="B27" s="4">
         <f>SUM(B4:B26)</f>
-        <v>674.5</v>
+        <v>790.05</v>
       </c>
       <c r="C27" s="4">
         <f>SUM(C4:C26)</f>
-        <v>627.25</v>
+        <v>871.75</v>
       </c>
       <c r="D27" s="4">
         <f>SUM(D4:D26)</f>
-        <v>580.25</v>
+        <v>824.5</v>
       </c>
       <c r="E27" s="4">
         <f>SUM(E4:E26)</f>
-        <v>568.04999999999995</v>
+        <v>711.8</v>
       </c>
       <c r="F27" s="4">
         <f>SUM(F4:F26)</f>
-        <v>603.25</v>
+        <v>726</v>
       </c>
       <c r="G27" s="4">
-        <f>SUM(B27:F27)</f>
-        <v>3053.3</v>
+        <f t="shared" si="0"/>
+        <v>3924.1000000000004</v>
       </c>
     </row>
   </sheetData>
@@ -2593,13 +2693,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>62</v>
       </c>
@@ -2610,86 +2710,98 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>41</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>63</v>
       </c>
       <c r="B4" s="8">
-        <v>78</v>
+        <f>78+10</f>
+        <v>88</v>
       </c>
       <c r="C4" s="8">
-        <v>73</v>
+        <f>73+20</f>
+        <v>93</v>
       </c>
       <c r="D4" s="8">
-        <v>67</v>
+        <f>67+22</f>
+        <v>89</v>
       </c>
       <c r="E4" s="8">
-        <v>58</v>
+        <f>58+25</f>
+        <v>83</v>
       </c>
       <c r="F4" s="8">
-        <v>90</v>
+        <f>90+16</f>
+        <v>106</v>
       </c>
       <c r="G4" s="7">
-        <f>SUM(B4:F4)</f>
-        <v>366</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" ref="G4:G10" si="0">SUM(B4:F4)</f>
+        <v>459</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>64</v>
       </c>
       <c r="B5" s="8">
-        <v>27</v>
+        <f>27+3</f>
+        <v>30</v>
       </c>
       <c r="C5" s="8">
-        <v>14</v>
+        <f>14+3</f>
+        <v>17</v>
       </c>
       <c r="D5" s="8">
-        <v>18</v>
+        <f>18+2</f>
+        <v>20</v>
       </c>
       <c r="E5" s="8">
-        <v>15</v>
+        <f>1+15</f>
+        <v>16</v>
       </c>
       <c r="F5" s="8">
-        <v>10</v>
+        <f>10+1</f>
+        <v>11</v>
       </c>
       <c r="G5" s="7">
-        <f>SUM(B5:F5)</f>
-        <v>84</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>66</v>
       </c>
       <c r="B6" s="8">
-        <v>4</v>
+        <f>4+3</f>
+        <v>7</v>
       </c>
       <c r="C6" s="8">
-        <v>13</v>
+        <f>13+1</f>
+        <v>14</v>
       </c>
       <c r="D6" s="8">
         <v>4</v>
@@ -2701,33 +2813,36 @@
         <v>13</v>
       </c>
       <c r="G6" s="7">
-        <f>SUM(B6:F6)</f>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>65</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8">
-        <v>5</v>
+        <f>5+1</f>
+        <v>6</v>
       </c>
       <c r="D7" s="8">
         <v>3</v>
       </c>
-      <c r="E7" s="8"/>
+      <c r="E7" s="8">
+        <v>1</v>
+      </c>
       <c r="F7" s="8">
         <v>1</v>
       </c>
       <c r="G7" s="7">
-        <f>SUM(B7:F7)</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B8" s="8">
         <v>3</v>
@@ -2741,13 +2856,13 @@
         <v>2</v>
       </c>
       <c r="G8" s="7">
-        <f>SUM(B8:F8)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -2757,37 +2872,37 @@
         <v>1</v>
       </c>
       <c r="G9" s="7">
-        <f>SUM(B9:F9)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>54</v>
       </c>
       <c r="B10" s="4">
         <f>SUM(B4:B9)</f>
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="C10" s="4">
         <f>SUM(C4:C9)</f>
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="D10" s="4">
         <f>SUM(D4:D9)</f>
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="E10" s="4">
         <f>SUM(E4:E9)</f>
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="F10" s="4">
         <f>SUM(F4:F9)</f>
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="G10" s="4">
-        <f>SUM(B10:F10)</f>
-        <v>517</v>
+        <f t="shared" si="0"/>
+        <v>626</v>
       </c>
     </row>
   </sheetData>
@@ -2801,14 +2916,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>67</v>
       </c>
@@ -2818,29 +2933,29 @@
       <c r="E1" s="12"/>
       <c r="F1" s="12"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>68</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>69</v>
+        <v>110</v>
       </c>
       <c r="B4" s="8">
         <v>2.0299999999999998</v>
@@ -2858,23 +2973,43 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B5" s="17">
-        <f>AVERAGE(B4:F4)</f>
-        <v>2.1520000000000001</v>
-      </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="8">
+        <v>2.06</v>
+      </c>
+      <c r="C5" s="8">
+        <v>1.84</v>
+      </c>
+      <c r="D5" s="8">
+        <v>1.63</v>
+      </c>
+      <c r="E5" s="8">
+        <v>1.7</v>
+      </c>
+      <c r="F5" s="8">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="17">
+        <f>AVERAGE(B4:F5)</f>
+        <v>1.9590000000000001</v>
+      </c>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2884,15 +3019,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -2901,75 +3036,81 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>68</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B4" s="8">
-        <v>25</v>
+        <f>25+1</f>
+        <v>26</v>
       </c>
       <c r="C4" s="8">
         <v>21</v>
       </c>
       <c r="D4" s="8">
-        <v>22</v>
+        <f>22+1</f>
+        <v>23</v>
       </c>
       <c r="E4" s="8">
-        <v>7</v>
+        <f>7+1</f>
+        <v>8</v>
       </c>
       <c r="F4" s="8">
         <v>19</v>
       </c>
       <c r="G4" s="7">
         <f>SUM(B4:F4)</f>
-        <v>94</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B5" s="8">
-        <v>13.75</v>
+        <f>13.75+11.5</f>
+        <v>25.25</v>
       </c>
       <c r="C5" s="8">
         <v>23.25</v>
       </c>
       <c r="D5" s="8">
-        <v>19</v>
+        <f>19+15.5</f>
+        <v>34.5</v>
       </c>
       <c r="E5" s="8">
-        <v>5</v>
+        <f>5+26</f>
+        <v>31</v>
       </c>
       <c r="F5" s="8">
         <v>12.25</v>
       </c>
       <c r="G5" s="7">
         <f>SUM(B5:F5)</f>
-        <v>73.25</v>
+        <v>126.25</v>
       </c>
     </row>
   </sheetData>
@@ -2984,11 +3125,11 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B72C5E1-D8EF-BD4B-9990-2660E94F2C3D}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -2997,30 +3138,30 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B4" s="8">
         <v>2</v>

</xml_diff>

<commit_message>
Actualizar datos.xlsx con datos corregidos YTD Mayo 2026 (#17)
Total trabajos: 517 → 616 (+99 trabajos, +19%)
Total horas: 3.053h → 3.924h (+871h, +29%)
Retail: nueva categoría con volumen significativo (99 proyectos, 748h)
Entrega: nueva estructura con desglose Bdesign/Retail (media 1.96d vs 2.15d)
RRSS: 94 → 97 publicaciones, 73h → 126h
Actualiza parseExcel para leer hoja Entrega con múltiples categorías

https://claude.ai/code/session_01A4SLDFHLc22bTWoXT2NUrv

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos.xlsx
+++ b/datos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscar.nieto/Desktop/T/BDESIGN/DASHBOARD/__INTERACTIVO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://savillsglobal-my.sharepoint.com/personal/oscar_nieto_savills_es/Documents/Archivos de chat de Microsoft Teams/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A89D243B-7CED-E64E-BDFF-E29013313185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="132" documentId="13_ncr:1_{A89D243B-7CED-E64E-BDFF-E29013313185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94ADA68F-4576-43E6-92A7-705F8C539229}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="3264" yWindow="2664" windowWidth="17436" windowHeight="9756" tabRatio="500" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="111">
   <si>
     <t>PLANTILLA DASHBOARD BDESIGN</t>
   </si>
@@ -252,9 +252,6 @@
     <t>Métrica</t>
   </si>
   <si>
-    <t>Días medios de entrega</t>
-  </si>
-  <si>
     <t>MEDIA YTD</t>
   </si>
   <si>
@@ -376,6 +373,9 @@
   </si>
   <si>
     <t>Sevilla</t>
+  </si>
+  <si>
+    <t>Bdesign</t>
   </si>
 </sst>
 </file>
@@ -524,14 +524,14 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -620,6 +620,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -802,262 +806,277 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D37"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="4" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="23" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:4" ht="22.8" x14ac:dyDescent="0.4">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-    </row>
-    <row r="3" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+    </row>
+    <row r="3" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-    </row>
-    <row r="6" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+    </row>
+    <row r="6" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-    </row>
-    <row r="7" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+    </row>
+    <row r="7" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-    </row>
-    <row r="9" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+    </row>
+    <row r="9" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-    </row>
-    <row r="12" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+    </row>
+    <row r="12" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-    </row>
-    <row r="13" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+    </row>
+    <row r="13" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-    </row>
-    <row r="14" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+    </row>
+    <row r="14" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="15" t="s">
+      <c r="B14" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-    </row>
-    <row r="15" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+    </row>
+    <row r="15" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-    </row>
-    <row r="16" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+    </row>
+    <row r="16" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="15" t="s">
+      <c r="B16" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-    </row>
-    <row r="17" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+    </row>
+    <row r="17" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="15" t="s">
+      <c r="B17" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-    </row>
-    <row r="20" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+    </row>
+    <row r="20" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="15" t="s">
+      <c r="B22" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-    </row>
-    <row r="23" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+    </row>
+    <row r="23" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="B23" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-    </row>
-    <row r="24" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+    </row>
+    <row r="24" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-    </row>
-    <row r="25" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+    </row>
+    <row r="25" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-    </row>
-    <row r="26" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+    </row>
+    <row r="26" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B26" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-    </row>
-    <row r="29" spans="1:4" ht="18" x14ac:dyDescent="0.2">
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+    </row>
+    <row r="29" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-    </row>
-    <row r="32" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+    </row>
+    <row r="32" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="15" t="s">
+      <c r="B32" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-    </row>
-    <row r="33" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+    </row>
+    <row r="33" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B33" s="15" t="s">
+      <c r="B33" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C33" s="15"/>
-      <c r="D33" s="15"/>
-    </row>
-    <row r="34" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+    </row>
+    <row r="34" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B34" s="15" t="s">
+      <c r="B34" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-    </row>
-    <row r="35" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+    </row>
+    <row r="35" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B35" s="15" t="s">
+      <c r="B35" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-    </row>
-    <row r="36" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+    </row>
+    <row r="36" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B36" s="15" t="s">
+      <c r="B36" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
-    </row>
-    <row r="37" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+    </row>
+    <row r="37" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B37" s="15" t="s">
+      <c r="B37" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C37" s="15"/>
-      <c r="D37" s="15"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B25:D25"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="B37:D37"/>
@@ -1066,21 +1085,6 @@
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1090,13 +1094,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>47</v>
       </c>
@@ -1107,78 +1111,86 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>48</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>50</v>
       </c>
       <c r="B4" s="8">
-        <v>23</v>
+        <f>23+7</f>
+        <v>30</v>
       </c>
       <c r="C4" s="8">
-        <v>28</v>
+        <f>28+10</f>
+        <v>38</v>
       </c>
       <c r="D4" s="8">
-        <v>23</v>
+        <f>23+8</f>
+        <v>31</v>
       </c>
       <c r="E4" s="8">
-        <v>25</v>
+        <f>25+9</f>
+        <v>34</v>
       </c>
       <c r="F4" s="8">
-        <v>38</v>
+        <f>38+8</f>
+        <v>46</v>
       </c>
       <c r="G4" s="9">
-        <f>SUM(B4:F4)</f>
-        <v>137</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" ref="G4:G18" si="0">SUM(B4:F4)</f>
+        <v>179</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>45</v>
       </c>
       <c r="B5" s="8">
-        <v>25</v>
+        <f>25+1</f>
+        <v>26</v>
       </c>
       <c r="C5" s="8">
         <v>21</v>
       </c>
       <c r="D5" s="8">
-        <v>22</v>
+        <f>22+1</f>
+        <v>23</v>
       </c>
       <c r="E5" s="8">
-        <v>7</v>
+        <f>7+1</f>
+        <v>8</v>
       </c>
       <c r="F5" s="8">
         <v>20</v>
       </c>
       <c r="G5" s="9">
-        <f>SUM(B5:F5)</f>
-        <v>95</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>51</v>
       </c>
@@ -1192,52 +1204,62 @@
         <v>12</v>
       </c>
       <c r="E6" s="8">
-        <v>13</v>
+        <f>13+2</f>
+        <v>15</v>
       </c>
       <c r="F6" s="8">
-        <v>18</v>
+        <f>18+1</f>
+        <v>19</v>
       </c>
       <c r="G6" s="9">
-        <f>SUM(B6:F6)</f>
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B7" s="8">
+        <f>14+2</f>
+        <v>16</v>
+      </c>
+      <c r="C7" s="8">
+        <f>8+6</f>
         <v>14</v>
       </c>
-      <c r="C7" s="8">
-        <v>8</v>
-      </c>
       <c r="D7" s="8">
-        <v>11</v>
+        <f>11+3</f>
+        <v>14</v>
       </c>
       <c r="E7" s="8">
-        <v>11</v>
+        <f>11+10</f>
+        <v>21</v>
       </c>
       <c r="F7" s="8">
-        <v>12</v>
+        <f>12+4</f>
+        <v>16</v>
       </c>
       <c r="G7" s="9">
-        <f>SUM(B7:F7)</f>
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>52</v>
       </c>
       <c r="B8" s="8">
+        <f>9+1</f>
+        <v>10</v>
+      </c>
+      <c r="C8" s="8">
+        <f>6+1</f>
+        <v>7</v>
+      </c>
+      <c r="D8" s="8">
+        <f>7+2</f>
         <v>9</v>
-      </c>
-      <c r="C8" s="8">
-        <v>6</v>
-      </c>
-      <c r="D8" s="8">
-        <v>7</v>
       </c>
       <c r="E8" s="8">
         <v>11</v>
@@ -1246,13 +1268,13 @@
         <v>3</v>
       </c>
       <c r="G8" s="9">
-        <f>SUM(B8:F8)</f>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B9" s="8">
         <v>5</v>
@@ -1270,13 +1292,13 @@
         <v>3</v>
       </c>
       <c r="G9" s="9">
-        <f>SUM(B9:F9)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B10" s="8">
         <v>3</v>
@@ -1294,37 +1316,42 @@
         <v>8</v>
       </c>
       <c r="G10" s="9">
-        <f>SUM(B10:F10)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B11" s="8">
-        <v>9</v>
+        <f>9+1</f>
+        <v>10</v>
       </c>
       <c r="C11" s="8">
+        <f>4+6</f>
+        <v>10</v>
+      </c>
+      <c r="D11" s="8">
+        <f>4+3</f>
+        <v>7</v>
+      </c>
+      <c r="E11" s="8">
+        <f>3+2</f>
+        <v>5</v>
+      </c>
+      <c r="F11" s="8">
+        <f>3+1</f>
         <v>4</v>
       </c>
-      <c r="D11" s="8">
-        <v>4</v>
-      </c>
-      <c r="E11" s="8">
-        <v>3</v>
-      </c>
-      <c r="F11" s="8">
-        <v>3</v>
-      </c>
       <c r="G11" s="9">
-        <f>SUM(B11:F11)</f>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B12" s="8">
         <v>3</v>
@@ -1332,24 +1359,30 @@
       <c r="C12" s="8">
         <v>1</v>
       </c>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
+      <c r="D12" s="8">
+        <v>0</v>
+      </c>
+      <c r="E12" s="8">
+        <v>0</v>
+      </c>
       <c r="F12" s="8">
         <v>7</v>
       </c>
       <c r="G12" s="9">
-        <f>SUM(B12:F12)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>53</v>
       </c>
       <c r="B13" s="8">
         <v>4</v>
       </c>
-      <c r="C13" s="8"/>
+      <c r="C13" s="8">
+        <v>0</v>
+      </c>
       <c r="D13" s="8">
         <v>1</v>
       </c>
@@ -1360,16 +1393,17 @@
         <v>2</v>
       </c>
       <c r="G13" s="9">
-        <f>SUM(B13:F13)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B14" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="C14" s="8">
         <v>2</v>
@@ -1382,93 +1416,113 @@
         <v>2</v>
       </c>
       <c r="G14" s="9">
-        <f>SUM(B14:F14)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B15" s="8">
+        <f>2+1</f>
+        <v>3</v>
+      </c>
+      <c r="C15" s="8">
+        <f>2+1</f>
+        <v>3</v>
+      </c>
+      <c r="D15" s="8">
+        <f>2+1</f>
+        <v>3</v>
+      </c>
+      <c r="E15" s="8">
+        <v>1</v>
+      </c>
+      <c r="F15" s="8">
+        <v>0</v>
+      </c>
+      <c r="G15" s="9">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="8" t="s">
         <v>78</v>
-      </c>
-      <c r="B15" s="8">
-        <v>2</v>
-      </c>
-      <c r="C15" s="8">
-        <v>2</v>
-      </c>
-      <c r="D15" s="8">
-        <v>2</v>
-      </c>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="9">
-        <f>SUM(B15:F15)</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="8" t="s">
-        <v>79</v>
       </c>
       <c r="B16" s="8">
         <v>3</v>
       </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
+      <c r="C16" s="8">
+        <v>0</v>
+      </c>
+      <c r="D16" s="8">
+        <v>2</v>
+      </c>
       <c r="E16" s="8">
         <v>1</v>
       </c>
       <c r="F16" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="G16" s="9">
-        <f>SUM(B16:F16)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
+        <v>81</v>
+      </c>
+      <c r="B17" s="8">
+        <v>0</v>
+      </c>
+      <c r="C17" s="8">
+        <v>0</v>
+      </c>
+      <c r="D17" s="8">
+        <v>1</v>
+      </c>
       <c r="E17" s="8">
         <v>1</v>
       </c>
-      <c r="F17" s="8"/>
+      <c r="F17" s="8">
+        <v>0</v>
+      </c>
       <c r="G17" s="10">
-        <f>SUM(B17:F17)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>54</v>
       </c>
       <c r="B18" s="11">
         <f>SUM(B4:B17)</f>
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C18" s="11">
         <f>SUM(C4:C17)</f>
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="D18" s="11">
         <f>SUM(D4:D17)</f>
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="E18" s="11">
         <f>SUM(E4:E17)</f>
-        <v>89</v>
+        <v>114</v>
       </c>
       <c r="F18" s="11">
         <f>SUM(F4:F17)</f>
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="G18" s="11">
-        <f>SUM(B18:F18)</f>
-        <v>517</v>
+        <f t="shared" si="0"/>
+        <v>616</v>
       </c>
     </row>
   </sheetData>
@@ -1483,13 +1537,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>55</v>
       </c>
@@ -1500,35 +1554,36 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>56</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B4" s="8">
-        <v>26</v>
+        <f>26+1</f>
+        <v>27</v>
       </c>
       <c r="C4" s="8">
         <v>24</v>
@@ -1537,17 +1592,19 @@
         <v>20</v>
       </c>
       <c r="E4" s="8">
+        <f>18+2</f>
+        <v>20</v>
+      </c>
+      <c r="F4" s="8">
+        <f>15+3</f>
         <v>18</v>
       </c>
-      <c r="F4" s="8">
-        <v>15</v>
-      </c>
       <c r="G4" s="8">
-        <f>SUM(B4:F4)</f>
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" ref="G4:G25" si="0">SUM(B4:F4)</f>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>57</v>
       </c>
@@ -1567,13 +1624,13 @@
         <v>36</v>
       </c>
       <c r="G5" s="8">
-        <f>SUM(B5:F5)</f>
+        <f t="shared" si="0"/>
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B6" s="8">
         <v>14</v>
@@ -1591,13 +1648,13 @@
         <v>9</v>
       </c>
       <c r="G6" s="8">
-        <f>SUM(B6:F6)</f>
+        <f t="shared" si="0"/>
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B7" s="8">
         <v>7</v>
@@ -1609,17 +1666,18 @@
         <v>16</v>
       </c>
       <c r="E7" s="8">
-        <v>13</v>
+        <f>13+1</f>
+        <v>14</v>
       </c>
       <c r="F7" s="8">
         <v>1</v>
       </c>
       <c r="G7" s="8">
-        <f>SUM(B7:F7)</f>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>58</v>
       </c>
@@ -1627,7 +1685,8 @@
         <v>10</v>
       </c>
       <c r="C8" s="8">
-        <v>10</v>
+        <f>10+1</f>
+        <v>11</v>
       </c>
       <c r="D8" s="8">
         <v>5</v>
@@ -1639,13 +1698,13 @@
         <v>6</v>
       </c>
       <c r="G8" s="8">
-        <f>SUM(B8:F8)</f>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B9" s="8">
         <v>5</v>
@@ -1663,13 +1722,13 @@
         <v>17</v>
       </c>
       <c r="G9" s="8">
-        <f>SUM(B9:F9)</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B10" s="8">
         <v>12</v>
@@ -1687,22 +1746,24 @@
         <v>3</v>
       </c>
       <c r="G10" s="8">
-        <f>SUM(B10:F10)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B11" s="8">
-        <v>5</v>
+        <f>5+1</f>
+        <v>6</v>
       </c>
       <c r="C11" s="8">
         <v>4</v>
       </c>
       <c r="D11" s="8">
-        <v>5</v>
+        <f>5+2</f>
+        <v>7</v>
       </c>
       <c r="E11" s="8">
         <v>3</v>
@@ -1711,11 +1772,11 @@
         <v>7</v>
       </c>
       <c r="G11" s="8">
-        <f>SUM(B11:F11)</f>
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>60</v>
       </c>
@@ -1735,57 +1796,65 @@
         <v>7</v>
       </c>
       <c r="G12" s="8">
-        <f>SUM(B12:F12)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>59</v>
       </c>
       <c r="B13" s="8">
-        <v>3</v>
+        <f>3+12</f>
+        <v>15</v>
       </c>
       <c r="C13" s="8">
-        <v>2</v>
+        <f>2+23</f>
+        <v>25</v>
       </c>
       <c r="D13" s="8">
-        <v>3</v>
-      </c>
-      <c r="E13" s="8"/>
+        <f>3+18</f>
+        <v>21</v>
+      </c>
+      <c r="E13" s="8">
+        <v>23</v>
+      </c>
       <c r="F13" s="8">
-        <v>2</v>
+        <f>2+13</f>
+        <v>15</v>
       </c>
       <c r="G13" s="8">
-        <f>SUM(B13:F13)</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8">
         <v>3</v>
       </c>
       <c r="D14" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="E14" s="8">
         <v>1</v>
       </c>
       <c r="F14" s="8">
-        <v>3</v>
+        <f>3+1</f>
+        <v>4</v>
       </c>
       <c r="G14" s="8">
-        <f>SUM(B14:F14)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8">
@@ -1799,35 +1868,39 @@
         <v>3</v>
       </c>
       <c r="G15" s="8">
-        <f>SUM(B15:F15)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B16" s="8">
-        <v>1</v>
+        <f>1+2</f>
+        <v>3</v>
       </c>
       <c r="C16" s="8">
         <v>2</v>
       </c>
-      <c r="D16" s="8"/>
+      <c r="D16" s="8">
+        <v>2</v>
+      </c>
       <c r="E16" s="8">
         <v>3</v>
       </c>
       <c r="F16" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="G16" s="8">
-        <f>SUM(B16:F16)</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B17" s="8">
         <v>3</v>
@@ -1841,19 +1914,20 @@
         <v>2</v>
       </c>
       <c r="G17" s="8">
-        <f>SUM(B17:F17)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B18" s="8">
         <v>2</v>
       </c>
       <c r="C18" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="D18" s="8">
         <v>1</v>
@@ -1863,13 +1937,13 @@
       </c>
       <c r="F18" s="8"/>
       <c r="G18" s="8">
-        <f>SUM(B18:F18)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="8">
@@ -1883,13 +1957,13 @@
         <v>2</v>
       </c>
       <c r="G19" s="8">
-        <f>SUM(B19:F19)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B20" s="8">
         <v>1</v>
@@ -1905,13 +1979,13 @@
         <v>1</v>
       </c>
       <c r="G20" s="8">
-        <f>SUM(B20:F20)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8">
@@ -1923,13 +1997,13 @@
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
       <c r="G21" s="8">
-        <f>SUM(B21:F21)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -1939,31 +2013,34 @@
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
       <c r="G22" s="8">
-        <f>SUM(B22:F22)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
       <c r="D23" s="8">
         <v>1</v>
       </c>
-      <c r="E23" s="8"/>
+      <c r="E23" s="8">
+        <v>1</v>
+      </c>
       <c r="F23" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="G23" s="8">
-        <f>SUM(B23:F23)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B24" s="8">
         <v>1</v>
@@ -1973,37 +2050,37 @@
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
       <c r="G24" s="8">
-        <f>SUM(B24:F24)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>54</v>
       </c>
       <c r="B25" s="4">
         <f>SUM(B4:B24)</f>
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="C25" s="4">
         <f>SUM(C4:C24)</f>
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="D25" s="4">
         <f>SUM(D4:D24)</f>
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="E25" s="4">
         <f>SUM(E4:E24)</f>
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="F25" s="4">
         <f>SUM(F4:F24)</f>
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="G25" s="4">
-        <f>SUM(B25:F25)</f>
-        <v>517</v>
+        <f t="shared" si="0"/>
+        <v>627</v>
       </c>
     </row>
   </sheetData>
@@ -2018,13 +2095,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>61</v>
       </c>
@@ -2035,35 +2112,36 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>56</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B4" s="8">
-        <v>165.5</v>
+        <f>165.5+0.5</f>
+        <v>166</v>
       </c>
       <c r="C4" s="8">
         <v>279.75</v>
@@ -2078,11 +2156,11 @@
         <v>191</v>
       </c>
       <c r="G4" s="7">
-        <f>SUM(B4:F4)</f>
-        <v>923.25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" ref="G4:G27" si="0">SUM(B4:F4)</f>
+        <v>923.75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>57</v>
       </c>
@@ -2102,13 +2180,13 @@
         <v>110.25</v>
       </c>
       <c r="G5" s="7">
-        <f>SUM(B5:F5)</f>
+        <f t="shared" si="0"/>
         <v>399.55</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B6" s="8">
         <v>26.5</v>
@@ -2120,17 +2198,19 @@
         <v>102.5</v>
       </c>
       <c r="E6" s="8">
-        <v>58</v>
+        <f>58+9.5</f>
+        <v>67.5</v>
       </c>
       <c r="F6" s="8">
-        <v>25.75</v>
+        <f>25.75+7.5</f>
+        <v>33.25</v>
       </c>
       <c r="G6" s="7">
-        <f>SUM(B6:F6)</f>
-        <v>275</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>292</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>58</v>
       </c>
@@ -2138,7 +2218,8 @@
         <v>89</v>
       </c>
       <c r="C7" s="8">
-        <v>65.5</v>
+        <f>65.5+3</f>
+        <v>68.5</v>
       </c>
       <c r="D7" s="8">
         <v>28</v>
@@ -2150,13 +2231,13 @@
         <v>19.75</v>
       </c>
       <c r="G7" s="7">
-        <f>SUM(B7:F7)</f>
-        <v>268.25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>271.25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B8" s="8">
         <v>29.25</v>
@@ -2168,19 +2249,20 @@
         <v>71.5</v>
       </c>
       <c r="E8" s="8">
-        <v>81</v>
+        <f>81+3</f>
+        <v>84</v>
       </c>
       <c r="F8" s="8">
         <v>1</v>
       </c>
       <c r="G8" s="7">
-        <f>SUM(B8:F8)</f>
-        <v>226.25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>229.25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B9" s="8">
         <v>74</v>
@@ -2198,13 +2280,13 @@
         <v>24.75</v>
       </c>
       <c r="G9" s="7">
-        <f>SUM(B9:F9)</f>
+        <f t="shared" si="0"/>
         <v>182.75</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B10" s="8">
         <v>13</v>
@@ -2222,22 +2304,24 @@
         <v>82</v>
       </c>
       <c r="G10" s="7">
-        <f>SUM(B10:F10)</f>
+        <f t="shared" si="0"/>
         <v>171.5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B11" s="8">
-        <v>16.75</v>
+        <f>16.75+20.5</f>
+        <v>37.25</v>
       </c>
       <c r="C11" s="8">
         <v>8</v>
       </c>
       <c r="D11" s="8">
-        <v>38</v>
+        <f>38+31.5</f>
+        <v>69.5</v>
       </c>
       <c r="E11" s="8">
         <v>40.5</v>
@@ -2246,11 +2330,11 @@
         <v>37.5</v>
       </c>
       <c r="G11" s="7">
-        <f>SUM(B11:F11)</f>
-        <v>140.75</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>192.75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>60</v>
       </c>
@@ -2270,13 +2354,13 @@
         <v>32.5</v>
       </c>
       <c r="G12" s="7">
-        <f>SUM(B12:F12)</f>
+        <f t="shared" si="0"/>
         <v>106.75</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B13" s="8">
         <v>9</v>
@@ -2294,13 +2378,13 @@
         <v>5</v>
       </c>
       <c r="G13" s="7">
-        <f>SUM(B13:F13)</f>
+        <f t="shared" si="0"/>
         <v>62.75</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8">
@@ -2314,13 +2398,13 @@
         <v>48</v>
       </c>
       <c r="G14" s="7">
-        <f>SUM(B14:F14)</f>
+        <f t="shared" si="0"/>
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B15" s="8">
         <v>39.5</v>
@@ -2334,13 +2418,13 @@
         <v>4.5</v>
       </c>
       <c r="G15" s="7">
-        <f>SUM(B15:F15)</f>
+        <f t="shared" si="0"/>
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B16" s="8">
         <v>4.5</v>
@@ -2356,79 +2440,91 @@
         <v>4</v>
       </c>
       <c r="G16" s="7">
-        <f>SUM(B16:F16)</f>
+        <f t="shared" si="0"/>
         <v>27.75</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>59</v>
       </c>
       <c r="B17" s="8">
-        <v>13.5</v>
+        <f>13.5+72.55</f>
+        <v>86.05</v>
       </c>
       <c r="C17" s="8">
-        <v>3.75</v>
+        <f>3.75+240.5</f>
+        <v>244.25</v>
       </c>
       <c r="D17" s="8">
-        <v>5.75</v>
-      </c>
-      <c r="E17" s="8"/>
+        <f>5.75+207.5</f>
+        <v>213.25</v>
+      </c>
+      <c r="E17" s="8">
+        <v>125.25</v>
+      </c>
       <c r="F17" s="8">
-        <v>4</v>
+        <f>4+75</f>
+        <v>79</v>
       </c>
       <c r="G17" s="7">
-        <f>SUM(B17:F17)</f>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>747.8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="8">
         <v>14.5</v>
       </c>
       <c r="D18" s="8">
-        <v>5</v>
+        <f>5+1</f>
+        <v>6</v>
       </c>
       <c r="E18" s="8">
         <v>4</v>
       </c>
       <c r="F18" s="8">
-        <v>3.25</v>
+        <f>3.25+27.5</f>
+        <v>30.75</v>
       </c>
       <c r="G18" s="7">
-        <f>SUM(B18:F18)</f>
-        <v>26.75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>55.25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B19" s="8">
-        <v>3</v>
+        <f>3+22</f>
+        <v>25</v>
       </c>
       <c r="C19" s="8">
         <v>4</v>
       </c>
-      <c r="D19" s="8"/>
+      <c r="D19" s="8">
+        <v>4.25</v>
+      </c>
       <c r="E19" s="8">
         <v>16.75</v>
       </c>
       <c r="F19" s="8">
-        <v>1</v>
+        <f>1+1.25</f>
+        <v>2.25</v>
       </c>
       <c r="G19" s="7">
-        <f>SUM(B19:F19)</f>
-        <v>24.75</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>52.25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -2438,31 +2534,34 @@
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
       <c r="G20" s="7">
-        <f>SUM(B20:F20)</f>
+        <f t="shared" si="0"/>
         <v>24.25</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
       <c r="D21" s="8">
         <v>13</v>
       </c>
-      <c r="E21" s="8"/>
+      <c r="E21" s="8">
+        <v>6</v>
+      </c>
       <c r="F21" s="8">
-        <v>3</v>
+        <f>3+11.5</f>
+        <v>14.5</v>
       </c>
       <c r="G21" s="7">
-        <f>SUM(B21:F21)</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B22" s="8">
         <v>12</v>
@@ -2472,13 +2571,13 @@
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
       <c r="G22" s="7">
-        <f>SUM(B22:F22)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8">
@@ -2490,13 +2589,13 @@
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
       <c r="G23" s="7">
-        <f>SUM(B23:F23)</f>
+        <f t="shared" si="0"/>
         <v>11.5</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8">
@@ -2510,19 +2609,20 @@
         <v>5</v>
       </c>
       <c r="G24" s="7">
-        <f>SUM(B24:F24)</f>
+        <f t="shared" si="0"/>
         <v>9.5</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B25" s="8">
         <v>5</v>
       </c>
       <c r="C25" s="8">
-        <v>1</v>
+        <f>1+1</f>
+        <v>2</v>
       </c>
       <c r="D25" s="8">
         <v>1</v>
@@ -2532,13 +2632,13 @@
       </c>
       <c r="F25" s="8"/>
       <c r="G25" s="7">
-        <f>SUM(B25:F25)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -2548,37 +2648,37 @@
         <v>1</v>
       </c>
       <c r="G26" s="7">
-        <f>SUM(B26:F26)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>54</v>
       </c>
       <c r="B27" s="4">
         <f>SUM(B4:B26)</f>
-        <v>674.5</v>
+        <v>790.05</v>
       </c>
       <c r="C27" s="4">
         <f>SUM(C4:C26)</f>
-        <v>627.25</v>
+        <v>871.75</v>
       </c>
       <c r="D27" s="4">
         <f>SUM(D4:D26)</f>
-        <v>580.25</v>
+        <v>824.5</v>
       </c>
       <c r="E27" s="4">
         <f>SUM(E4:E26)</f>
-        <v>568.04999999999995</v>
+        <v>711.8</v>
       </c>
       <c r="F27" s="4">
         <f>SUM(F4:F26)</f>
-        <v>603.25</v>
+        <v>726</v>
       </c>
       <c r="G27" s="4">
-        <f>SUM(B27:F27)</f>
-        <v>3053.3</v>
+        <f t="shared" si="0"/>
+        <v>3924.1000000000004</v>
       </c>
     </row>
   </sheetData>
@@ -2593,13 +2693,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>62</v>
       </c>
@@ -2610,86 +2710,98 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>41</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>63</v>
       </c>
       <c r="B4" s="8">
-        <v>78</v>
+        <f>78+10</f>
+        <v>88</v>
       </c>
       <c r="C4" s="8">
-        <v>73</v>
+        <f>73+20</f>
+        <v>93</v>
       </c>
       <c r="D4" s="8">
-        <v>67</v>
+        <f>67+22</f>
+        <v>89</v>
       </c>
       <c r="E4" s="8">
-        <v>58</v>
+        <f>58+25</f>
+        <v>83</v>
       </c>
       <c r="F4" s="8">
-        <v>90</v>
+        <f>90+16</f>
+        <v>106</v>
       </c>
       <c r="G4" s="7">
-        <f>SUM(B4:F4)</f>
-        <v>366</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" ref="G4:G10" si="0">SUM(B4:F4)</f>
+        <v>459</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>64</v>
       </c>
       <c r="B5" s="8">
-        <v>27</v>
+        <f>27+3</f>
+        <v>30</v>
       </c>
       <c r="C5" s="8">
-        <v>14</v>
+        <f>14+3</f>
+        <v>17</v>
       </c>
       <c r="D5" s="8">
-        <v>18</v>
+        <f>18+2</f>
+        <v>20</v>
       </c>
       <c r="E5" s="8">
-        <v>15</v>
+        <f>1+15</f>
+        <v>16</v>
       </c>
       <c r="F5" s="8">
-        <v>10</v>
+        <f>10+1</f>
+        <v>11</v>
       </c>
       <c r="G5" s="7">
-        <f>SUM(B5:F5)</f>
-        <v>84</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>66</v>
       </c>
       <c r="B6" s="8">
-        <v>4</v>
+        <f>4+3</f>
+        <v>7</v>
       </c>
       <c r="C6" s="8">
-        <v>13</v>
+        <f>13+1</f>
+        <v>14</v>
       </c>
       <c r="D6" s="8">
         <v>4</v>
@@ -2701,33 +2813,36 @@
         <v>13</v>
       </c>
       <c r="G6" s="7">
-        <f>SUM(B6:F6)</f>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>65</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8">
-        <v>5</v>
+        <f>5+1</f>
+        <v>6</v>
       </c>
       <c r="D7" s="8">
         <v>3</v>
       </c>
-      <c r="E7" s="8"/>
+      <c r="E7" s="8">
+        <v>1</v>
+      </c>
       <c r="F7" s="8">
         <v>1</v>
       </c>
       <c r="G7" s="7">
-        <f>SUM(B7:F7)</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B8" s="8">
         <v>3</v>
@@ -2741,13 +2856,13 @@
         <v>2</v>
       </c>
       <c r="G8" s="7">
-        <f>SUM(B8:F8)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -2757,37 +2872,37 @@
         <v>1</v>
       </c>
       <c r="G9" s="7">
-        <f>SUM(B9:F9)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>54</v>
       </c>
       <c r="B10" s="4">
         <f>SUM(B4:B9)</f>
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="C10" s="4">
         <f>SUM(C4:C9)</f>
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="D10" s="4">
         <f>SUM(D4:D9)</f>
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="E10" s="4">
         <f>SUM(E4:E9)</f>
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="F10" s="4">
         <f>SUM(F4:F9)</f>
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="G10" s="4">
-        <f>SUM(B10:F10)</f>
-        <v>517</v>
+        <f t="shared" si="0"/>
+        <v>626</v>
       </c>
     </row>
   </sheetData>
@@ -2801,14 +2916,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>67</v>
       </c>
@@ -2818,29 +2933,29 @@
       <c r="E1" s="12"/>
       <c r="F1" s="12"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>68</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>69</v>
+        <v>110</v>
       </c>
       <c r="B4" s="8">
         <v>2.0299999999999998</v>
@@ -2858,23 +2973,43 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B5" s="17">
-        <f>AVERAGE(B4:F4)</f>
-        <v>2.1520000000000001</v>
-      </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="8">
+        <v>2.06</v>
+      </c>
+      <c r="C5" s="8">
+        <v>1.84</v>
+      </c>
+      <c r="D5" s="8">
+        <v>1.63</v>
+      </c>
+      <c r="E5" s="8">
+        <v>1.7</v>
+      </c>
+      <c r="F5" s="8">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="17">
+        <f>AVERAGE(B4:F5)</f>
+        <v>1.9590000000000001</v>
+      </c>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2884,15 +3019,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -2901,75 +3036,81 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>68</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B4" s="8">
-        <v>25</v>
+        <f>25+1</f>
+        <v>26</v>
       </c>
       <c r="C4" s="8">
         <v>21</v>
       </c>
       <c r="D4" s="8">
-        <v>22</v>
+        <f>22+1</f>
+        <v>23</v>
       </c>
       <c r="E4" s="8">
-        <v>7</v>
+        <f>7+1</f>
+        <v>8</v>
       </c>
       <c r="F4" s="8">
         <v>19</v>
       </c>
       <c r="G4" s="7">
         <f>SUM(B4:F4)</f>
-        <v>94</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B5" s="8">
-        <v>13.75</v>
+        <f>13.75+11.5</f>
+        <v>25.25</v>
       </c>
       <c r="C5" s="8">
         <v>23.25</v>
       </c>
       <c r="D5" s="8">
-        <v>19</v>
+        <f>19+15.5</f>
+        <v>34.5</v>
       </c>
       <c r="E5" s="8">
-        <v>5</v>
+        <f>5+26</f>
+        <v>31</v>
       </c>
       <c r="F5" s="8">
         <v>12.25</v>
       </c>
       <c r="G5" s="7">
         <f>SUM(B5:F5)</f>
-        <v>73.25</v>
+        <v>126.25</v>
       </c>
     </row>
   </sheetData>
@@ -2984,11 +3125,11 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B72C5E1-D8EF-BD4B-9990-2660E94F2C3D}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -2997,30 +3138,30 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
       <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B4" s="8">
         <v>2</v>

</xml_diff>